<commit_message>
Store orders and upload spreadsheet are disjoint order sets
populate_shop now creates orders-only by default (Shiv's store already has
products; --products for a fresh store) selling the store's own premium wall;
the xlsx becomes the shop's other-channel (eBay/Depop) sales — zero overlapping
line items, so connect + upload merge without double-counting.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/streetwear_vault_orders.xlsx
+++ b/backend/data/streetwear_vault_orders.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 01:41:41 +0100</t>
+          <t>2026-07-11 01:49:59 +0100</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-09 23:41:41 +0100</t>
+          <t>2026-07-09 23:49:59 +0100</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-07 19:41:41 +0100</t>
+          <t>2026-07-07 19:49:59 +0100</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-06 19:41:41 +0100</t>
+          <t>2026-07-06 19:49:59 +0100</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-05 01:41:41 +0100</t>
+          <t>2026-07-05 01:49:59 +0100</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-04 14:41:41 +0100</t>
+          <t>2026-07-04 14:49:59 +0100</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-02 19:41:41 +0100</t>
+          <t>2026-07-02 19:49:59 +0100</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-30 21:41:41 +0100</t>
+          <t>2026-06-30 21:49:59 +0100</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-30 15:41:41 +0100</t>
+          <t>2026-06-30 15:49:59 +0100</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-30 15:41:41 +0100</t>
+          <t>2026-06-30 15:49:59 +0100</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-29 13:41:41 +0100</t>
+          <t>2026-06-29 13:49:59 +0100</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-27 06:41:41 +0100</t>
+          <t>2026-06-27 06:49:59 +0100</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-26 21:41:41 +0100</t>
+          <t>2026-06-26 21:49:59 +0100</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -960,16 +960,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-23 13:41:41 +0100</t>
+          <t>2026-06-23 13:49:59 +0100</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New Balance 550 - White/Green</t>
+          <t>New Balance 2002R - Protection Pack</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>91.66</v>
+        <v>119.78</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
@@ -998,7 +998,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-21 08:41:41 +0100</t>
+          <t>2026-06-21 08:49:59 +0100</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-20 18:41:41 +0100</t>
+          <t>2026-06-20 18:49:59 +0100</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-18 05:41:41 +0100</t>
+          <t>2026-06-18 05:49:59 +0100</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-17 13:41:41 +0100</t>
+          <t>2026-06-17 13:49:59 +0100</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1150,12 +1150,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-17 03:41:41 +0100</t>
+          <t>2026-06-17 03:49:59 +0100</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Carhartt WIP Michigan Chore Coat - Black</t>
+          <t>Carhartt WIP OG Chore Coat - Dearborn</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-13 18:41:41 +0100</t>
+          <t>2026-06-13 18:49:59 +0100</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-13 03:41:41 +0100</t>
+          <t>2026-06-13 03:49:59 +0100</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-13 01:41:41 +0100</t>
+          <t>2026-06-13 01:49:59 +0100</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-12 11:41:41 +0100</t>
+          <t>2026-06-12 11:49:59 +0100</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-12 08:41:41 +0100</t>
+          <t>2026-06-12 08:49:59 +0100</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-07 22:41:41 +0100</t>
+          <t>2026-06-07 22:49:59 +0100</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-06 11:41:41 +0100</t>
+          <t>2026-06-06 11:49:59 +0100</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-05 20:41:41 +0100</t>
+          <t>2026-06-05 20:49:59 +0100</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-05 10:41:41 +0100</t>
+          <t>2026-06-05 10:49:59 +0100</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-03 21:41:41 +0100</t>
+          <t>2026-06-03 21:49:59 +0100</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-30 13:41:41 +0100</t>
+          <t>2026-05-30 13:49:59 +0100</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-29 20:41:41 +0100</t>
+          <t>2026-05-29 20:49:59 +0100</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-28 21:41:41 +0100</t>
+          <t>2026-05-28 21:49:59 +0100</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-28 08:41:41 +0100</t>
+          <t>2026-05-28 08:49:59 +0100</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-05-24 03:41:41 +0100</t>
+          <t>2026-05-24 03:49:59 +0100</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-05-21 19:41:41 +0100</t>
+          <t>2026-05-21 19:49:59 +0100</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-20 14:41:41 +0100</t>
+          <t>2026-05-20 14:49:59 +0100</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1834,12 +1834,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-19 07:41:41 +0100</t>
+          <t>2026-05-19 07:49:59 +0100</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Carhartt WIP Michigan Chore Coat - Black</t>
+          <t>Carhartt WIP OG Chore Coat - Dearborn</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-18 03:41:41 +0100</t>
+          <t>2026-05-18 03:49:59 +0100</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-15 08:41:41 +0100</t>
+          <t>2026-05-15 08:49:59 +0100</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-14 09:41:41 +0100</t>
+          <t>2026-05-14 09:49:59 +0100</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-14 02:41:41 +0100</t>
+          <t>2026-05-14 02:49:59 +0100</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2024,23 +2024,23 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-13 23:41:41 +0100</t>
+          <t>2026-05-13 23:49:59 +0100</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>The North Face Nuptse 700 - Black</t>
+          <t>Salomon XT-6 - Black/Phantom</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>112.21</v>
+        <v>98.18000000000001</v>
       </c>
       <c r="E43" t="n">
         <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>The North Face</t>
+          <t>Salomon</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2062,16 +2062,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-13 08:41:41 +0100</t>
+          <t>2026-05-13 08:49:59 +0100</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>New Balance 550 - White/Green</t>
+          <t>New Balance 2002R - Protection Pack</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>80.26000000000001</v>
+        <v>104.89</v>
       </c>
       <c r="E44" t="n">
         <v>1</v>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-11 15:41:41 +0100</t>
+          <t>2026-05-11 15:49:59 +0100</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-05-09 04:41:41 +0100</t>
+          <t>2026-05-09 04:49:59 +0100</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-05-06 23:41:41 +0100</t>
+          <t>2026-05-06 23:49:59 +0100</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-05-06 18:41:41 +0100</t>
+          <t>2026-05-06 18:49:59 +0100</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-05-05 11:41:41 +0100</t>
+          <t>2026-05-05 11:49:59 +0100</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">

</xml_diff>